<commit_message>
Enhance Historical PO Import Functionality
- Updated the historical PO import process to include commissioning details, ensuring imported POs are marked as commissioned with the appropriate date and user.
- Revised documentation to reflect changes in the import requirements, including the need for `commissioned_at` and `commissioned_by` fields.
- Improved the KA historical PO template to clarify the handling of `external_po_ref`, `brand_name`, and `rfpf_number` across multiple lines.
- Enhanced the import scripts to support the new commissioning logic and ensure accurate data processing during imports.
</commit_message>
<xml_diff>
--- a/docs/KA_Historical_PO_Fill_Template.xlsx
+++ b/docs/KA_Historical_PO_Fill_Template.xlsx
@@ -1,1424 +1,1432 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0261CB46-C4DE-40B6-A3C5-B412B873FA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Read_Me" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="PO_Lines" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Column_Guide" state="visible" r:id="rId6"/>
+    <sheet name="Read_Me" sheetId="1" r:id="rId1"/>
+    <sheet name="PO_Lines" sheetId="2" r:id="rId2"/>
+    <sheet name="Column_Guide" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="O1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U1" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="A2" authorId="0">
+    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+      <text/>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+      <text/>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
+      <text/>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
+      <text/>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
+      <text/>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
+      <text/>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007000000}">
+      <text/>
+    </comment>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000008000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Old PO number. Repeat on every line of the same PO.</t>
         </r>
       </text>
     </comment>
-    <comment ref="B2" authorId="0">
+    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000009000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Real 2024 date. YYYY-MM-DD. Not the day you type it.</t>
         </r>
       </text>
     </comment>
-    <comment ref="C2" authorId="0">
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000A000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Client name as in OMS (or close). Agent matches to client_code.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D2" authorId="0">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000B000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Required if the client has more than one shop.</t>
         </r>
       </text>
     </comment>
-    <comment ref="E2" authorId="0">
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000C000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Required if the shop has more than one delivery address.</t>
         </r>
       </text>
     </comment>
-    <comment ref="F2" authorId="0">
+    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000D000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Hub warehouse brand. Same variant name can exist on another brand — always fill both.</t>
         </r>
       </text>
     </comment>
-    <comment ref="G2" authorId="0">
+    <comment ref="G2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000E000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Hub warehouse variant name. Matched with brand_name, never variant name alone.</t>
         </r>
       </text>
     </comment>
-    <comment ref="H2" authorId="0">
+    <comment ref="H2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000F000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Units on this line.</t>
         </r>
       </text>
     </comment>
-    <comment ref="I2" authorId="0">
+    <comment ref="I2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000010000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Price per unit.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J2" authorId="0">
+    <comment ref="J2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000011000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Optional. Leave blank to use quantity × unit_price.</t>
         </r>
       </text>
     </comment>
-    <comment ref="K2" authorId="0">
+    <comment ref="K2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000012000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>KAM / owner email in OMS. Recommended.</t>
         </r>
       </text>
     </comment>
-    <comment ref="L2" authorId="0">
+    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000013000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Leave blank to use linked main warehouse.</t>
         </r>
       </text>
     </comment>
-    <comment ref="M2" authorId="0">
+    <comment ref="M2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000014000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>PO header discount. Default 0. Repeat same value on every line of the PO.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N2" authorId="0">
+    <comment ref="N2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000015000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>PO header RFPF. Repeat the same value on every line of the PO. Leave blank if none.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O2" authorId="0">
+    <comment ref="O2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000016000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>Optional. Legacy ref is added automatically.</t>
         </r>
       </text>
     </comment>
-    <comment ref="P2" authorId="0">
+    <comment ref="P2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000017000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>LEAVE BLANK. Agent fills from hub brand + variant.</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q2" authorId="0">
+    <comment ref="Q2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000018000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>LEAVE BLANK. Agent fills from client_name.</t>
         </r>
       </text>
     </comment>
-    <comment ref="R2" authorId="0">
+    <comment ref="R2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000019000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>LEAVE BLANK. Agent fills from shop_name.</t>
         </r>
       </text>
     </comment>
-    <comment ref="S2" authorId="0">
+    <comment ref="S2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001A000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>LEAVE BLANK. Importer sets full PO total (treat as paid).</t>
         </r>
       </text>
     </comment>
-    <comment ref="T2" authorId="0">
+    <comment ref="T2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001B000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>LEAVE BLANK. Defaults to CASH.</t>
         </r>
       </text>
     </comment>
-    <comment ref="U2" authorId="0">
+    <comment ref="U2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001C000000}">
       <text>
         <r>
           <rPr>
+            <sz val="11"/>
             <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
             <scheme val="minor"/>
-            <sz val="11"/>
-            <rFont val="Calibri"/>
           </rPr>
           <t>LEAVE BLANK. Defaults to order_date.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U3" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U4" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U5" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U6" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U7" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U8" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U9" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U10" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U11" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U12" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U13" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U14" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U15" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U16" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U17" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U18" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U19" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U20" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U21" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U22" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U23" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U24" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U25" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U26" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U27" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U28" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U29" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U30" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U31" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U32" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U33" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U34" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U35" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U36" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U37" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U38" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U39" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U40" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U41" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U42" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U43" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U44" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U45" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U46" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U47" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U48" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U49" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U50" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U51" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U52" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U53" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="O54" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="P54" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="Q54" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="R54" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="S54" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="T54" authorId="0">
-      <text/>
-    </comment>
-    <comment ref="U54" authorId="0">
+    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001D000000}">
+      <text/>
+    </comment>
+    <comment ref="P3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001E000000}">
+      <text/>
+    </comment>
+    <comment ref="Q3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001F000000}">
+      <text/>
+    </comment>
+    <comment ref="R3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000020000000}">
+      <text/>
+    </comment>
+    <comment ref="S3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000021000000}">
+      <text/>
+    </comment>
+    <comment ref="T3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000022000000}">
+      <text/>
+    </comment>
+    <comment ref="U3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000023000000}">
+      <text/>
+    </comment>
+    <comment ref="O4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000024000000}">
+      <text/>
+    </comment>
+    <comment ref="P4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000025000000}">
+      <text/>
+    </comment>
+    <comment ref="Q4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000026000000}">
+      <text/>
+    </comment>
+    <comment ref="R4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000027000000}">
+      <text/>
+    </comment>
+    <comment ref="S4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000028000000}">
+      <text/>
+    </comment>
+    <comment ref="T4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000029000000}">
+      <text/>
+    </comment>
+    <comment ref="U4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002A000000}">
+      <text/>
+    </comment>
+    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002B000000}">
+      <text/>
+    </comment>
+    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002C000000}">
+      <text/>
+    </comment>
+    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002D000000}">
+      <text/>
+    </comment>
+    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002E000000}">
+      <text/>
+    </comment>
+    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002F000000}">
+      <text/>
+    </comment>
+    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000030000000}">
+      <text/>
+    </comment>
+    <comment ref="U5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000031000000}">
+      <text/>
+    </comment>
+    <comment ref="O6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000032000000}">
+      <text/>
+    </comment>
+    <comment ref="P6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000033000000}">
+      <text/>
+    </comment>
+    <comment ref="Q6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000034000000}">
+      <text/>
+    </comment>
+    <comment ref="R6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000035000000}">
+      <text/>
+    </comment>
+    <comment ref="S6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000036000000}">
+      <text/>
+    </comment>
+    <comment ref="T6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000037000000}">
+      <text/>
+    </comment>
+    <comment ref="U6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000038000000}">
+      <text/>
+    </comment>
+    <comment ref="O7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000039000000}">
+      <text/>
+    </comment>
+    <comment ref="P7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003A000000}">
+      <text/>
+    </comment>
+    <comment ref="Q7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003B000000}">
+      <text/>
+    </comment>
+    <comment ref="R7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003C000000}">
+      <text/>
+    </comment>
+    <comment ref="S7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003D000000}">
+      <text/>
+    </comment>
+    <comment ref="T7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003E000000}">
+      <text/>
+    </comment>
+    <comment ref="U7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003F000000}">
+      <text/>
+    </comment>
+    <comment ref="O8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000040000000}">
+      <text/>
+    </comment>
+    <comment ref="P8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000041000000}">
+      <text/>
+    </comment>
+    <comment ref="Q8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000042000000}">
+      <text/>
+    </comment>
+    <comment ref="R8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000043000000}">
+      <text/>
+    </comment>
+    <comment ref="S8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000044000000}">
+      <text/>
+    </comment>
+    <comment ref="T8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000045000000}">
+      <text/>
+    </comment>
+    <comment ref="U8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000046000000}">
+      <text/>
+    </comment>
+    <comment ref="O9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000047000000}">
+      <text/>
+    </comment>
+    <comment ref="P9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000048000000}">
+      <text/>
+    </comment>
+    <comment ref="Q9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000049000000}">
+      <text/>
+    </comment>
+    <comment ref="R9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004A000000}">
+      <text/>
+    </comment>
+    <comment ref="S9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004B000000}">
+      <text/>
+    </comment>
+    <comment ref="T9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004C000000}">
+      <text/>
+    </comment>
+    <comment ref="U9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004D000000}">
+      <text/>
+    </comment>
+    <comment ref="O10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004E000000}">
+      <text/>
+    </comment>
+    <comment ref="P10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004F000000}">
+      <text/>
+    </comment>
+    <comment ref="Q10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000050000000}">
+      <text/>
+    </comment>
+    <comment ref="R10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000051000000}">
+      <text/>
+    </comment>
+    <comment ref="S10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000052000000}">
+      <text/>
+    </comment>
+    <comment ref="T10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000053000000}">
+      <text/>
+    </comment>
+    <comment ref="U10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000054000000}">
+      <text/>
+    </comment>
+    <comment ref="O11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000055000000}">
+      <text/>
+    </comment>
+    <comment ref="P11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000056000000}">
+      <text/>
+    </comment>
+    <comment ref="Q11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000057000000}">
+      <text/>
+    </comment>
+    <comment ref="R11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000058000000}">
+      <text/>
+    </comment>
+    <comment ref="S11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000059000000}">
+      <text/>
+    </comment>
+    <comment ref="T11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005A000000}">
+      <text/>
+    </comment>
+    <comment ref="U11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005B000000}">
+      <text/>
+    </comment>
+    <comment ref="O12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005C000000}">
+      <text/>
+    </comment>
+    <comment ref="P12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005D000000}">
+      <text/>
+    </comment>
+    <comment ref="Q12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005E000000}">
+      <text/>
+    </comment>
+    <comment ref="R12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005F000000}">
+      <text/>
+    </comment>
+    <comment ref="S12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000060000000}">
+      <text/>
+    </comment>
+    <comment ref="T12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000061000000}">
+      <text/>
+    </comment>
+    <comment ref="U12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000062000000}">
+      <text/>
+    </comment>
+    <comment ref="O13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000063000000}">
+      <text/>
+    </comment>
+    <comment ref="P13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000064000000}">
+      <text/>
+    </comment>
+    <comment ref="Q13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000065000000}">
+      <text/>
+    </comment>
+    <comment ref="R13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000066000000}">
+      <text/>
+    </comment>
+    <comment ref="S13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000067000000}">
+      <text/>
+    </comment>
+    <comment ref="T13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000068000000}">
+      <text/>
+    </comment>
+    <comment ref="U13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000069000000}">
+      <text/>
+    </comment>
+    <comment ref="O14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006A000000}">
+      <text/>
+    </comment>
+    <comment ref="P14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006B000000}">
+      <text/>
+    </comment>
+    <comment ref="Q14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006C000000}">
+      <text/>
+    </comment>
+    <comment ref="R14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006D000000}">
+      <text/>
+    </comment>
+    <comment ref="S14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006E000000}">
+      <text/>
+    </comment>
+    <comment ref="T14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006F000000}">
+      <text/>
+    </comment>
+    <comment ref="U14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000070000000}">
+      <text/>
+    </comment>
+    <comment ref="O15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000071000000}">
+      <text/>
+    </comment>
+    <comment ref="P15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000072000000}">
+      <text/>
+    </comment>
+    <comment ref="Q15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000073000000}">
+      <text/>
+    </comment>
+    <comment ref="R15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000074000000}">
+      <text/>
+    </comment>
+    <comment ref="S15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000075000000}">
+      <text/>
+    </comment>
+    <comment ref="T15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000076000000}">
+      <text/>
+    </comment>
+    <comment ref="U15" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000077000000}">
+      <text/>
+    </comment>
+    <comment ref="O16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000078000000}">
+      <text/>
+    </comment>
+    <comment ref="P16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000079000000}">
+      <text/>
+    </comment>
+    <comment ref="Q16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007A000000}">
+      <text/>
+    </comment>
+    <comment ref="R16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007B000000}">
+      <text/>
+    </comment>
+    <comment ref="S16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007C000000}">
+      <text/>
+    </comment>
+    <comment ref="T16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007D000000}">
+      <text/>
+    </comment>
+    <comment ref="U16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007E000000}">
+      <text/>
+    </comment>
+    <comment ref="O17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007F000000}">
+      <text/>
+    </comment>
+    <comment ref="P17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000080000000}">
+      <text/>
+    </comment>
+    <comment ref="Q17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000081000000}">
+      <text/>
+    </comment>
+    <comment ref="R17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000082000000}">
+      <text/>
+    </comment>
+    <comment ref="S17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000083000000}">
+      <text/>
+    </comment>
+    <comment ref="T17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000084000000}">
+      <text/>
+    </comment>
+    <comment ref="U17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000085000000}">
+      <text/>
+    </comment>
+    <comment ref="O18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000086000000}">
+      <text/>
+    </comment>
+    <comment ref="P18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000087000000}">
+      <text/>
+    </comment>
+    <comment ref="Q18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000088000000}">
+      <text/>
+    </comment>
+    <comment ref="R18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000089000000}">
+      <text/>
+    </comment>
+    <comment ref="S18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00008A000000}">
+      <text/>
+    </comment>
+    <comment ref="T18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00008B000000}">
+      <text/>
+    </comment>
+    <comment ref="U18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00008C000000}">
+      <text/>
+    </comment>
+    <comment ref="O19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00008D000000}">
+      <text/>
+    </comment>
+    <comment ref="P19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00008E000000}">
+      <text/>
+    </comment>
+    <comment ref="Q19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00008F000000}">
+      <text/>
+    </comment>
+    <comment ref="R19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000090000000}">
+      <text/>
+    </comment>
+    <comment ref="S19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000091000000}">
+      <text/>
+    </comment>
+    <comment ref="T19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000092000000}">
+      <text/>
+    </comment>
+    <comment ref="U19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000093000000}">
+      <text/>
+    </comment>
+    <comment ref="O20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000094000000}">
+      <text/>
+    </comment>
+    <comment ref="P20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000095000000}">
+      <text/>
+    </comment>
+    <comment ref="Q20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000096000000}">
+      <text/>
+    </comment>
+    <comment ref="R20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000097000000}">
+      <text/>
+    </comment>
+    <comment ref="S20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000098000000}">
+      <text/>
+    </comment>
+    <comment ref="T20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000099000000}">
+      <text/>
+    </comment>
+    <comment ref="U20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00009A000000}">
+      <text/>
+    </comment>
+    <comment ref="O21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00009B000000}">
+      <text/>
+    </comment>
+    <comment ref="P21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00009C000000}">
+      <text/>
+    </comment>
+    <comment ref="Q21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00009D000000}">
+      <text/>
+    </comment>
+    <comment ref="R21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00009E000000}">
+      <text/>
+    </comment>
+    <comment ref="S21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00009F000000}">
+      <text/>
+    </comment>
+    <comment ref="T21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A0000000}">
+      <text/>
+    </comment>
+    <comment ref="U21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A1000000}">
+      <text/>
+    </comment>
+    <comment ref="O22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A2000000}">
+      <text/>
+    </comment>
+    <comment ref="P22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A3000000}">
+      <text/>
+    </comment>
+    <comment ref="Q22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A4000000}">
+      <text/>
+    </comment>
+    <comment ref="R22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A5000000}">
+      <text/>
+    </comment>
+    <comment ref="S22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A6000000}">
+      <text/>
+    </comment>
+    <comment ref="T22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A7000000}">
+      <text/>
+    </comment>
+    <comment ref="U22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A8000000}">
+      <text/>
+    </comment>
+    <comment ref="O23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000A9000000}">
+      <text/>
+    </comment>
+    <comment ref="P23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000AA000000}">
+      <text/>
+    </comment>
+    <comment ref="Q23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000AB000000}">
+      <text/>
+    </comment>
+    <comment ref="R23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000AC000000}">
+      <text/>
+    </comment>
+    <comment ref="S23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000AD000000}">
+      <text/>
+    </comment>
+    <comment ref="T23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000AE000000}">
+      <text/>
+    </comment>
+    <comment ref="U23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000AF000000}">
+      <text/>
+    </comment>
+    <comment ref="O24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B0000000}">
+      <text/>
+    </comment>
+    <comment ref="P24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B1000000}">
+      <text/>
+    </comment>
+    <comment ref="Q24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B2000000}">
+      <text/>
+    </comment>
+    <comment ref="R24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B3000000}">
+      <text/>
+    </comment>
+    <comment ref="S24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B4000000}">
+      <text/>
+    </comment>
+    <comment ref="T24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B5000000}">
+      <text/>
+    </comment>
+    <comment ref="U24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B6000000}">
+      <text/>
+    </comment>
+    <comment ref="O25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B7000000}">
+      <text/>
+    </comment>
+    <comment ref="P25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B8000000}">
+      <text/>
+    </comment>
+    <comment ref="Q25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000B9000000}">
+      <text/>
+    </comment>
+    <comment ref="R25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000BA000000}">
+      <text/>
+    </comment>
+    <comment ref="S25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000BB000000}">
+      <text/>
+    </comment>
+    <comment ref="T25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000BC000000}">
+      <text/>
+    </comment>
+    <comment ref="U25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000BD000000}">
+      <text/>
+    </comment>
+    <comment ref="O26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000BE000000}">
+      <text/>
+    </comment>
+    <comment ref="P26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000BF000000}">
+      <text/>
+    </comment>
+    <comment ref="Q26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C0000000}">
+      <text/>
+    </comment>
+    <comment ref="R26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C1000000}">
+      <text/>
+    </comment>
+    <comment ref="S26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C2000000}">
+      <text/>
+    </comment>
+    <comment ref="T26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C3000000}">
+      <text/>
+    </comment>
+    <comment ref="U26" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C4000000}">
+      <text/>
+    </comment>
+    <comment ref="O27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C5000000}">
+      <text/>
+    </comment>
+    <comment ref="P27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C6000000}">
+      <text/>
+    </comment>
+    <comment ref="Q27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C7000000}">
+      <text/>
+    </comment>
+    <comment ref="R27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C8000000}">
+      <text/>
+    </comment>
+    <comment ref="S27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000C9000000}">
+      <text/>
+    </comment>
+    <comment ref="T27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000CA000000}">
+      <text/>
+    </comment>
+    <comment ref="U27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000CB000000}">
+      <text/>
+    </comment>
+    <comment ref="O28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000CC000000}">
+      <text/>
+    </comment>
+    <comment ref="P28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000CD000000}">
+      <text/>
+    </comment>
+    <comment ref="Q28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000CE000000}">
+      <text/>
+    </comment>
+    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000CF000000}">
+      <text/>
+    </comment>
+    <comment ref="S28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D0000000}">
+      <text/>
+    </comment>
+    <comment ref="T28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D1000000}">
+      <text/>
+    </comment>
+    <comment ref="U28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D2000000}">
+      <text/>
+    </comment>
+    <comment ref="O29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D3000000}">
+      <text/>
+    </comment>
+    <comment ref="P29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D4000000}">
+      <text/>
+    </comment>
+    <comment ref="Q29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D5000000}">
+      <text/>
+    </comment>
+    <comment ref="R29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D6000000}">
+      <text/>
+    </comment>
+    <comment ref="S29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D7000000}">
+      <text/>
+    </comment>
+    <comment ref="T29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D8000000}">
+      <text/>
+    </comment>
+    <comment ref="U29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000D9000000}">
+      <text/>
+    </comment>
+    <comment ref="O30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000DA000000}">
+      <text/>
+    </comment>
+    <comment ref="P30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000DB000000}">
+      <text/>
+    </comment>
+    <comment ref="Q30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000DC000000}">
+      <text/>
+    </comment>
+    <comment ref="R30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000DD000000}">
+      <text/>
+    </comment>
+    <comment ref="S30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000DE000000}">
+      <text/>
+    </comment>
+    <comment ref="T30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000DF000000}">
+      <text/>
+    </comment>
+    <comment ref="U30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E0000000}">
+      <text/>
+    </comment>
+    <comment ref="O31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E1000000}">
+      <text/>
+    </comment>
+    <comment ref="P31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E2000000}">
+      <text/>
+    </comment>
+    <comment ref="Q31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E3000000}">
+      <text/>
+    </comment>
+    <comment ref="R31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E4000000}">
+      <text/>
+    </comment>
+    <comment ref="S31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E5000000}">
+      <text/>
+    </comment>
+    <comment ref="T31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E6000000}">
+      <text/>
+    </comment>
+    <comment ref="U31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E7000000}">
+      <text/>
+    </comment>
+    <comment ref="O32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E8000000}">
+      <text/>
+    </comment>
+    <comment ref="P32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000E9000000}">
+      <text/>
+    </comment>
+    <comment ref="Q32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000EA000000}">
+      <text/>
+    </comment>
+    <comment ref="R32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000EB000000}">
+      <text/>
+    </comment>
+    <comment ref="S32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000EC000000}">
+      <text/>
+    </comment>
+    <comment ref="T32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000ED000000}">
+      <text/>
+    </comment>
+    <comment ref="U32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000EE000000}">
+      <text/>
+    </comment>
+    <comment ref="O33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000EF000000}">
+      <text/>
+    </comment>
+    <comment ref="P33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F0000000}">
+      <text/>
+    </comment>
+    <comment ref="Q33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F1000000}">
+      <text/>
+    </comment>
+    <comment ref="R33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F2000000}">
+      <text/>
+    </comment>
+    <comment ref="S33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F3000000}">
+      <text/>
+    </comment>
+    <comment ref="T33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F4000000}">
+      <text/>
+    </comment>
+    <comment ref="U33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F5000000}">
+      <text/>
+    </comment>
+    <comment ref="O34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F6000000}">
+      <text/>
+    </comment>
+    <comment ref="P34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F7000000}">
+      <text/>
+    </comment>
+    <comment ref="Q34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F8000000}">
+      <text/>
+    </comment>
+    <comment ref="R34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000F9000000}">
+      <text/>
+    </comment>
+    <comment ref="S34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000FA000000}">
+      <text/>
+    </comment>
+    <comment ref="T34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000FB000000}">
+      <text/>
+    </comment>
+    <comment ref="U34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000FC000000}">
+      <text/>
+    </comment>
+    <comment ref="O35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000FD000000}">
+      <text/>
+    </comment>
+    <comment ref="P35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000FE000000}">
+      <text/>
+    </comment>
+    <comment ref="Q35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-0000FF000000}">
+      <text/>
+    </comment>
+    <comment ref="R35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000000010000}">
+      <text/>
+    </comment>
+    <comment ref="S35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001010000}">
+      <text/>
+    </comment>
+    <comment ref="T35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002010000}">
+      <text/>
+    </comment>
+    <comment ref="U35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003010000}">
+      <text/>
+    </comment>
+    <comment ref="O36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004010000}">
+      <text/>
+    </comment>
+    <comment ref="P36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005010000}">
+      <text/>
+    </comment>
+    <comment ref="Q36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006010000}">
+      <text/>
+    </comment>
+    <comment ref="R36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007010000}">
+      <text/>
+    </comment>
+    <comment ref="S36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000008010000}">
+      <text/>
+    </comment>
+    <comment ref="T36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000009010000}">
+      <text/>
+    </comment>
+    <comment ref="U36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000A010000}">
+      <text/>
+    </comment>
+    <comment ref="O37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000B010000}">
+      <text/>
+    </comment>
+    <comment ref="P37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000C010000}">
+      <text/>
+    </comment>
+    <comment ref="Q37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000D010000}">
+      <text/>
+    </comment>
+    <comment ref="R37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000E010000}">
+      <text/>
+    </comment>
+    <comment ref="S37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000F010000}">
+      <text/>
+    </comment>
+    <comment ref="T37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000010010000}">
+      <text/>
+    </comment>
+    <comment ref="U37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000011010000}">
+      <text/>
+    </comment>
+    <comment ref="O38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000012010000}">
+      <text/>
+    </comment>
+    <comment ref="P38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000013010000}">
+      <text/>
+    </comment>
+    <comment ref="Q38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000014010000}">
+      <text/>
+    </comment>
+    <comment ref="R38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000015010000}">
+      <text/>
+    </comment>
+    <comment ref="S38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000016010000}">
+      <text/>
+    </comment>
+    <comment ref="T38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000017010000}">
+      <text/>
+    </comment>
+    <comment ref="U38" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000018010000}">
+      <text/>
+    </comment>
+    <comment ref="O39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000019010000}">
+      <text/>
+    </comment>
+    <comment ref="P39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001A010000}">
+      <text/>
+    </comment>
+    <comment ref="Q39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001B010000}">
+      <text/>
+    </comment>
+    <comment ref="R39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001C010000}">
+      <text/>
+    </comment>
+    <comment ref="S39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001D010000}">
+      <text/>
+    </comment>
+    <comment ref="T39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001E010000}">
+      <text/>
+    </comment>
+    <comment ref="U39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00001F010000}">
+      <text/>
+    </comment>
+    <comment ref="O40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000020010000}">
+      <text/>
+    </comment>
+    <comment ref="P40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000021010000}">
+      <text/>
+    </comment>
+    <comment ref="Q40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000022010000}">
+      <text/>
+    </comment>
+    <comment ref="R40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000023010000}">
+      <text/>
+    </comment>
+    <comment ref="S40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000024010000}">
+      <text/>
+    </comment>
+    <comment ref="T40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000025010000}">
+      <text/>
+    </comment>
+    <comment ref="U40" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000026010000}">
+      <text/>
+    </comment>
+    <comment ref="O41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000027010000}">
+      <text/>
+    </comment>
+    <comment ref="P41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000028010000}">
+      <text/>
+    </comment>
+    <comment ref="Q41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000029010000}">
+      <text/>
+    </comment>
+    <comment ref="R41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002A010000}">
+      <text/>
+    </comment>
+    <comment ref="S41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002B010000}">
+      <text/>
+    </comment>
+    <comment ref="T41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002C010000}">
+      <text/>
+    </comment>
+    <comment ref="U41" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002D010000}">
+      <text/>
+    </comment>
+    <comment ref="O42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002E010000}">
+      <text/>
+    </comment>
+    <comment ref="P42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00002F010000}">
+      <text/>
+    </comment>
+    <comment ref="Q42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000030010000}">
+      <text/>
+    </comment>
+    <comment ref="R42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000031010000}">
+      <text/>
+    </comment>
+    <comment ref="S42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000032010000}">
+      <text/>
+    </comment>
+    <comment ref="T42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000033010000}">
+      <text/>
+    </comment>
+    <comment ref="U42" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000034010000}">
+      <text/>
+    </comment>
+    <comment ref="O43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000035010000}">
+      <text/>
+    </comment>
+    <comment ref="P43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000036010000}">
+      <text/>
+    </comment>
+    <comment ref="Q43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000037010000}">
+      <text/>
+    </comment>
+    <comment ref="R43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000038010000}">
+      <text/>
+    </comment>
+    <comment ref="S43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000039010000}">
+      <text/>
+    </comment>
+    <comment ref="T43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003A010000}">
+      <text/>
+    </comment>
+    <comment ref="U43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003B010000}">
+      <text/>
+    </comment>
+    <comment ref="O44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003C010000}">
+      <text/>
+    </comment>
+    <comment ref="P44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003D010000}">
+      <text/>
+    </comment>
+    <comment ref="Q44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003E010000}">
+      <text/>
+    </comment>
+    <comment ref="R44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00003F010000}">
+      <text/>
+    </comment>
+    <comment ref="S44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000040010000}">
+      <text/>
+    </comment>
+    <comment ref="T44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000041010000}">
+      <text/>
+    </comment>
+    <comment ref="U44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000042010000}">
+      <text/>
+    </comment>
+    <comment ref="O45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000043010000}">
+      <text/>
+    </comment>
+    <comment ref="P45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000044010000}">
+      <text/>
+    </comment>
+    <comment ref="Q45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000045010000}">
+      <text/>
+    </comment>
+    <comment ref="R45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000046010000}">
+      <text/>
+    </comment>
+    <comment ref="S45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000047010000}">
+      <text/>
+    </comment>
+    <comment ref="T45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000048010000}">
+      <text/>
+    </comment>
+    <comment ref="U45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000049010000}">
+      <text/>
+    </comment>
+    <comment ref="O46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004A010000}">
+      <text/>
+    </comment>
+    <comment ref="P46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004B010000}">
+      <text/>
+    </comment>
+    <comment ref="Q46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004C010000}">
+      <text/>
+    </comment>
+    <comment ref="R46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004D010000}">
+      <text/>
+    </comment>
+    <comment ref="S46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004E010000}">
+      <text/>
+    </comment>
+    <comment ref="T46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00004F010000}">
+      <text/>
+    </comment>
+    <comment ref="U46" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000050010000}">
+      <text/>
+    </comment>
+    <comment ref="O47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000051010000}">
+      <text/>
+    </comment>
+    <comment ref="P47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000052010000}">
+      <text/>
+    </comment>
+    <comment ref="Q47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000053010000}">
+      <text/>
+    </comment>
+    <comment ref="R47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000054010000}">
+      <text/>
+    </comment>
+    <comment ref="S47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000055010000}">
+      <text/>
+    </comment>
+    <comment ref="T47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000056010000}">
+      <text/>
+    </comment>
+    <comment ref="U47" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000057010000}">
+      <text/>
+    </comment>
+    <comment ref="O48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000058010000}">
+      <text/>
+    </comment>
+    <comment ref="P48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000059010000}">
+      <text/>
+    </comment>
+    <comment ref="Q48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005A010000}">
+      <text/>
+    </comment>
+    <comment ref="R48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005B010000}">
+      <text/>
+    </comment>
+    <comment ref="S48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005C010000}">
+      <text/>
+    </comment>
+    <comment ref="T48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005D010000}">
+      <text/>
+    </comment>
+    <comment ref="U48" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005E010000}">
+      <text/>
+    </comment>
+    <comment ref="O49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00005F010000}">
+      <text/>
+    </comment>
+    <comment ref="P49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000060010000}">
+      <text/>
+    </comment>
+    <comment ref="Q49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000061010000}">
+      <text/>
+    </comment>
+    <comment ref="R49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000062010000}">
+      <text/>
+    </comment>
+    <comment ref="S49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000063010000}">
+      <text/>
+    </comment>
+    <comment ref="T49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000064010000}">
+      <text/>
+    </comment>
+    <comment ref="U49" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000065010000}">
+      <text/>
+    </comment>
+    <comment ref="O50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000066010000}">
+      <text/>
+    </comment>
+    <comment ref="P50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000067010000}">
+      <text/>
+    </comment>
+    <comment ref="Q50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000068010000}">
+      <text/>
+    </comment>
+    <comment ref="R50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000069010000}">
+      <text/>
+    </comment>
+    <comment ref="S50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006A010000}">
+      <text/>
+    </comment>
+    <comment ref="T50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006B010000}">
+      <text/>
+    </comment>
+    <comment ref="U50" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006C010000}">
+      <text/>
+    </comment>
+    <comment ref="O51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006D010000}">
+      <text/>
+    </comment>
+    <comment ref="P51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006E010000}">
+      <text/>
+    </comment>
+    <comment ref="Q51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00006F010000}">
+      <text/>
+    </comment>
+    <comment ref="R51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000070010000}">
+      <text/>
+    </comment>
+    <comment ref="S51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000071010000}">
+      <text/>
+    </comment>
+    <comment ref="T51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000072010000}">
+      <text/>
+    </comment>
+    <comment ref="U51" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000073010000}">
+      <text/>
+    </comment>
+    <comment ref="O52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000074010000}">
+      <text/>
+    </comment>
+    <comment ref="P52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000075010000}">
+      <text/>
+    </comment>
+    <comment ref="Q52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000076010000}">
+      <text/>
+    </comment>
+    <comment ref="R52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000077010000}">
+      <text/>
+    </comment>
+    <comment ref="S52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000078010000}">
+      <text/>
+    </comment>
+    <comment ref="T52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000079010000}">
+      <text/>
+    </comment>
+    <comment ref="U52" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007A010000}">
+      <text/>
+    </comment>
+    <comment ref="O53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007B010000}">
+      <text/>
+    </comment>
+    <comment ref="P53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007C010000}">
+      <text/>
+    </comment>
+    <comment ref="Q53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007D010000}">
+      <text/>
+    </comment>
+    <comment ref="R53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007E010000}">
+      <text/>
+    </comment>
+    <comment ref="S53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00007F010000}">
+      <text/>
+    </comment>
+    <comment ref="T53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000080010000}">
+      <text/>
+    </comment>
+    <comment ref="U53" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000081010000}">
+      <text/>
+    </comment>
+    <comment ref="O54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000082010000}">
+      <text/>
+    </comment>
+    <comment ref="P54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000083010000}">
+      <text/>
+    </comment>
+    <comment ref="Q54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000084010000}">
+      <text/>
+    </comment>
+    <comment ref="R54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000085010000}">
+      <text/>
+    </comment>
+    <comment ref="S54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000086010000}">
+      <text/>
+    </comment>
+    <comment ref="T54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000087010000}">
+      <text/>
+    </comment>
+    <comment ref="U54" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000088010000}">
       <text/>
     </comment>
   </commentList>
@@ -1426,7 +1434,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="109">
   <si>
     <t>KA historical PO — fill-in template</t>
   </si>
@@ -1596,9 +1604,6 @@
     <t>payment_date</t>
   </si>
   <si>
-    <t>LEGACY-2024-001</t>
-  </si>
-  <si>
     <t>2024-06-10</t>
   </si>
   <si>
@@ -1614,18 +1619,12 @@
     <t>Chillax</t>
   </si>
   <si>
-    <t>COSMIC CRUSH</t>
-  </si>
-  <si>
     <t>keyaccount3@gmail.com</t>
   </si>
   <si>
     <t>Same PO, different brand — keep brand_name</t>
   </si>
   <si>
-    <t>LEGACY-2024-002</t>
-  </si>
-  <si>
     <t>KAM First Client</t>
   </si>
   <si>
@@ -1744,22 +1743,40 @@
   </si>
   <si>
     <t>Equals order_date so cash sits in the PO month, not today.</t>
+  </si>
+  <si>
+    <t>TWILIGHT WILLOW (BLACKCURRANT)</t>
+  </si>
+  <si>
+    <t>LUSH ICE WATERMELON ICE</t>
+  </si>
+  <si>
+    <t>RFPF-123</t>
+  </si>
+  <si>
+    <t>RFPF-456</t>
+  </si>
+  <si>
+    <t>RFPF-2024-007</t>
+  </si>
+  <si>
+    <t>RFPF-2024-008</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -1777,17 +1794,17 @@
     </font>
     <font>
       <b/>
+      <sz val="9"/>
       <color rgb="FF111827"/>
-      <sz val="9"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1832,17 +1849,25 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1912,6 +1937,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2251,15 +2279,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="92" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="24" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2267,7 +2295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="18" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -2275,7 +2303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="18" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2283,7 +2311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="18" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -2291,7 +2319,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="18" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
@@ -2299,7 +2327,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="18" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -2307,7 +2335,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="18" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>1</v>
       </c>
@@ -2315,7 +2343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="18" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -2323,7 +2351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="18" customHeight="1">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -2331,7 +2359,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="18" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -2339,7 +2367,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="18" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
@@ -2347,7 +2375,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="18" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
@@ -2355,7 +2383,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="18" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>19</v>
       </c>
@@ -2363,7 +2391,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="18" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
@@ -2371,7 +2399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="18" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>21</v>
       </c>
@@ -2379,7 +2407,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="18" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
@@ -2387,7 +2415,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="18" customHeight="1">
       <c r="A17" s="5" t="s">
         <v>25</v>
       </c>
@@ -2395,7 +2423,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="18" customHeight="1">
       <c r="A18" s="6" t="s">
         <v>27</v>
       </c>
@@ -2403,7 +2431,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="18" customHeight="1">
       <c r="A19" s="7" t="s">
         <v>29</v>
       </c>
@@ -2413,14 +2441,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U54"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -2438,7 +2466,7 @@
     <col min="20" max="20" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.05" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="22.05" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>31</v>
       </c>
@@ -2503,7 +2531,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" ht="31.95" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="31.95" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>35</v>
       </c>
@@ -2568,39 +2596,39 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21">
       <c r="A3" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="C3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="D3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="E3" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="F3" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="16" t="s">
-        <v>61</v>
-      </c>
       <c r="G3" s="16" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="H3" s="18">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I3" s="18">
         <v>100</v>
       </c>
       <c r="J3" s="18">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L3" s="16" t="s">
         <v>1</v>
@@ -2608,9 +2636,11 @@
       <c r="M3" s="18">
         <v>0</v>
       </c>
-      <c r="N3" s="16"/>
+      <c r="N3" s="16" t="s">
+        <v>105</v>
+      </c>
       <c r="O3" s="16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P3" s="16" t="s">
         <v>1</v>
@@ -2631,27 +2661,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="17">
-        <v>45453</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>62</v>
+    <row r="4" spans="1:21" ht="28.8">
+      <c r="A4" s="16"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="34" t="s">
+        <v>104</v>
       </c>
       <c r="H4" s="18">
         <v>5</v>
@@ -2663,7 +2681,7 @@
         <v>500</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L4" s="16" t="s">
         <v>1</v>
@@ -2673,7 +2691,7 @@
       </c>
       <c r="N4" s="16"/>
       <c r="O4" s="16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P4" s="16" t="s">
         <v>1</v>
@@ -2694,27 +2712,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21">
       <c r="A5" s="20" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="B5" s="21">
         <v>46272</v>
       </c>
       <c r="C5" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="G5" s="20" t="s">
         <v>67</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="G5" s="20" t="s">
-        <v>70</v>
       </c>
       <c r="H5" s="23">
         <v>10</v>
@@ -2726,15 +2744,17 @@
         <v>1500</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L5" s="22"/>
       <c r="M5" s="24">
         <v>0</v>
       </c>
-      <c r="N5" s="22"/>
+      <c r="N5" s="22" t="s">
+        <v>106</v>
+      </c>
       <c r="O5" s="26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="P5" s="27"/>
       <c r="Q5" s="27"/>
@@ -2743,7 +2763,7 @@
       <c r="T5" s="27"/>
       <c r="U5" s="27"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21">
       <c r="A6" s="20"/>
       <c r="B6" s="21"/>
       <c r="C6" s="20"/>
@@ -2766,7 +2786,7 @@
       <c r="T6" s="27"/>
       <c r="U6" s="27"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21">
       <c r="A7" s="20"/>
       <c r="B7" s="21"/>
       <c r="C7" s="20"/>
@@ -2789,7 +2809,7 @@
       <c r="T7" s="27"/>
       <c r="U7" s="27"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21">
       <c r="A8" s="20"/>
       <c r="B8" s="21"/>
       <c r="C8" s="20"/>
@@ -2812,7 +2832,7 @@
       <c r="T8" s="27"/>
       <c r="U8" s="27"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21">
       <c r="A9" s="20"/>
       <c r="B9" s="21"/>
       <c r="C9" s="20"/>
@@ -2835,7 +2855,7 @@
       <c r="T9" s="27"/>
       <c r="U9" s="27"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21">
       <c r="A10" s="20"/>
       <c r="B10" s="21"/>
       <c r="C10" s="20"/>
@@ -2858,7 +2878,7 @@
       <c r="T10" s="27"/>
       <c r="U10" s="27"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21">
       <c r="A11" s="20"/>
       <c r="B11" s="21"/>
       <c r="C11" s="20"/>
@@ -2881,7 +2901,7 @@
       <c r="T11" s="27"/>
       <c r="U11" s="27"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21">
       <c r="A12" s="20"/>
       <c r="B12" s="21"/>
       <c r="C12" s="20"/>
@@ -2904,7 +2924,7 @@
       <c r="T12" s="27"/>
       <c r="U12" s="27"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21">
       <c r="A13" s="20"/>
       <c r="B13" s="21"/>
       <c r="C13" s="20"/>
@@ -2927,7 +2947,7 @@
       <c r="T13" s="27"/>
       <c r="U13" s="27"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21">
       <c r="A14" s="20"/>
       <c r="B14" s="21"/>
       <c r="C14" s="20"/>
@@ -2950,7 +2970,7 @@
       <c r="T14" s="27"/>
       <c r="U14" s="27"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21">
       <c r="A15" s="20"/>
       <c r="B15" s="21"/>
       <c r="C15" s="20"/>
@@ -2973,7 +2993,7 @@
       <c r="T15" s="27"/>
       <c r="U15" s="27"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21">
       <c r="A16" s="20"/>
       <c r="B16" s="21"/>
       <c r="C16" s="20"/>
@@ -2996,7 +3016,7 @@
       <c r="T16" s="27"/>
       <c r="U16" s="27"/>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21">
       <c r="A17" s="20"/>
       <c r="B17" s="21"/>
       <c r="C17" s="20"/>
@@ -3019,7 +3039,7 @@
       <c r="T17" s="27"/>
       <c r="U17" s="27"/>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21">
       <c r="A18" s="20"/>
       <c r="B18" s="21"/>
       <c r="C18" s="20"/>
@@ -3042,7 +3062,7 @@
       <c r="T18" s="27"/>
       <c r="U18" s="27"/>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21">
       <c r="A19" s="20"/>
       <c r="B19" s="21"/>
       <c r="C19" s="20"/>
@@ -3065,7 +3085,7 @@
       <c r="T19" s="27"/>
       <c r="U19" s="27"/>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21">
       <c r="A20" s="20"/>
       <c r="B20" s="21"/>
       <c r="C20" s="20"/>
@@ -3088,7 +3108,7 @@
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21">
       <c r="A21" s="20"/>
       <c r="B21" s="21"/>
       <c r="C21" s="20"/>
@@ -3111,7 +3131,7 @@
       <c r="T21" s="27"/>
       <c r="U21" s="27"/>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21">
       <c r="A22" s="20"/>
       <c r="B22" s="21"/>
       <c r="C22" s="20"/>
@@ -3134,7 +3154,7 @@
       <c r="T22" s="27"/>
       <c r="U22" s="27"/>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21">
       <c r="A23" s="20"/>
       <c r="B23" s="21"/>
       <c r="C23" s="20"/>
@@ -3157,7 +3177,7 @@
       <c r="T23" s="27"/>
       <c r="U23" s="27"/>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21">
       <c r="A24" s="20"/>
       <c r="B24" s="21"/>
       <c r="C24" s="20"/>
@@ -3180,7 +3200,7 @@
       <c r="T24" s="27"/>
       <c r="U24" s="27"/>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21">
       <c r="A25" s="20"/>
       <c r="B25" s="21"/>
       <c r="C25" s="20"/>
@@ -3203,7 +3223,7 @@
       <c r="T25" s="27"/>
       <c r="U25" s="27"/>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21">
       <c r="A26" s="20"/>
       <c r="B26" s="21"/>
       <c r="C26" s="20"/>
@@ -3226,7 +3246,7 @@
       <c r="T26" s="27"/>
       <c r="U26" s="27"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21">
       <c r="A27" s="20"/>
       <c r="B27" s="21"/>
       <c r="C27" s="20"/>
@@ -3249,7 +3269,7 @@
       <c r="T27" s="27"/>
       <c r="U27" s="27"/>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21">
       <c r="A28" s="20"/>
       <c r="B28" s="21"/>
       <c r="C28" s="20"/>
@@ -3272,7 +3292,7 @@
       <c r="T28" s="27"/>
       <c r="U28" s="27"/>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21">
       <c r="A29" s="20"/>
       <c r="B29" s="21"/>
       <c r="C29" s="20"/>
@@ -3295,7 +3315,7 @@
       <c r="T29" s="27"/>
       <c r="U29" s="27"/>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21">
       <c r="A30" s="20"/>
       <c r="B30" s="21"/>
       <c r="C30" s="20"/>
@@ -3318,7 +3338,7 @@
       <c r="T30" s="27"/>
       <c r="U30" s="27"/>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21">
       <c r="A31" s="20"/>
       <c r="B31" s="21"/>
       <c r="C31" s="20"/>
@@ -3341,7 +3361,7 @@
       <c r="T31" s="27"/>
       <c r="U31" s="27"/>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21">
       <c r="A32" s="20"/>
       <c r="B32" s="21"/>
       <c r="C32" s="20"/>
@@ -3364,7 +3384,7 @@
       <c r="T32" s="27"/>
       <c r="U32" s="27"/>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21">
       <c r="A33" s="20"/>
       <c r="B33" s="21"/>
       <c r="C33" s="20"/>
@@ -3387,7 +3407,7 @@
       <c r="T33" s="27"/>
       <c r="U33" s="27"/>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21">
       <c r="A34" s="20"/>
       <c r="B34" s="21"/>
       <c r="C34" s="20"/>
@@ -3410,7 +3430,7 @@
       <c r="T34" s="27"/>
       <c r="U34" s="27"/>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21">
       <c r="A35" s="20"/>
       <c r="B35" s="21"/>
       <c r="C35" s="20"/>
@@ -3433,7 +3453,7 @@
       <c r="T35" s="27"/>
       <c r="U35" s="27"/>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21">
       <c r="A36" s="20"/>
       <c r="B36" s="21"/>
       <c r="C36" s="20"/>
@@ -3456,7 +3476,7 @@
       <c r="T36" s="27"/>
       <c r="U36" s="27"/>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21">
       <c r="A37" s="20"/>
       <c r="B37" s="21"/>
       <c r="C37" s="20"/>
@@ -3479,7 +3499,7 @@
       <c r="T37" s="27"/>
       <c r="U37" s="27"/>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21">
       <c r="A38" s="20"/>
       <c r="B38" s="21"/>
       <c r="C38" s="20"/>
@@ -3502,7 +3522,7 @@
       <c r="T38" s="27"/>
       <c r="U38" s="27"/>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21">
       <c r="A39" s="20"/>
       <c r="B39" s="21"/>
       <c r="C39" s="20"/>
@@ -3525,7 +3545,7 @@
       <c r="T39" s="27"/>
       <c r="U39" s="27"/>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21">
       <c r="A40" s="20"/>
       <c r="B40" s="21"/>
       <c r="C40" s="20"/>
@@ -3548,7 +3568,7 @@
       <c r="T40" s="27"/>
       <c r="U40" s="27"/>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21">
       <c r="A41" s="20"/>
       <c r="B41" s="21"/>
       <c r="C41" s="20"/>
@@ -3571,7 +3591,7 @@
       <c r="T41" s="27"/>
       <c r="U41" s="27"/>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21">
       <c r="A42" s="20"/>
       <c r="B42" s="21"/>
       <c r="C42" s="20"/>
@@ -3594,7 +3614,7 @@
       <c r="T42" s="27"/>
       <c r="U42" s="27"/>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21">
       <c r="A43" s="20"/>
       <c r="B43" s="21"/>
       <c r="C43" s="20"/>
@@ -3617,7 +3637,7 @@
       <c r="T43" s="27"/>
       <c r="U43" s="27"/>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21">
       <c r="A44" s="20"/>
       <c r="B44" s="21"/>
       <c r="C44" s="20"/>
@@ -3640,7 +3660,7 @@
       <c r="T44" s="27"/>
       <c r="U44" s="27"/>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21">
       <c r="A45" s="20"/>
       <c r="B45" s="21"/>
       <c r="C45" s="20"/>
@@ -3663,7 +3683,7 @@
       <c r="T45" s="27"/>
       <c r="U45" s="27"/>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21">
       <c r="A46" s="20"/>
       <c r="B46" s="21"/>
       <c r="C46" s="20"/>
@@ -3686,7 +3706,7 @@
       <c r="T46" s="27"/>
       <c r="U46" s="27"/>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21">
       <c r="A47" s="20"/>
       <c r="B47" s="21"/>
       <c r="C47" s="20"/>
@@ -3709,7 +3729,7 @@
       <c r="T47" s="27"/>
       <c r="U47" s="27"/>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21">
       <c r="A48" s="20"/>
       <c r="B48" s="21"/>
       <c r="C48" s="20"/>
@@ -3732,7 +3752,7 @@
       <c r="T48" s="27"/>
       <c r="U48" s="27"/>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21">
       <c r="A49" s="20"/>
       <c r="B49" s="21"/>
       <c r="C49" s="20"/>
@@ -3755,7 +3775,7 @@
       <c r="T49" s="27"/>
       <c r="U49" s="27"/>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21">
       <c r="A50" s="20"/>
       <c r="B50" s="21"/>
       <c r="C50" s="20"/>
@@ -3778,7 +3798,7 @@
       <c r="T50" s="27"/>
       <c r="U50" s="27"/>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21">
       <c r="A51" s="20"/>
       <c r="B51" s="21"/>
       <c r="C51" s="20"/>
@@ -3801,7 +3821,7 @@
       <c r="T51" s="27"/>
       <c r="U51" s="27"/>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21">
       <c r="A52" s="20"/>
       <c r="B52" s="21"/>
       <c r="C52" s="20"/>
@@ -3824,7 +3844,7 @@
       <c r="T52" s="27"/>
       <c r="U52" s="27"/>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21">
       <c r="A53" s="20"/>
       <c r="B53" s="21"/>
       <c r="C53" s="20"/>
@@ -3847,7 +3867,7 @@
       <c r="T53" s="27"/>
       <c r="U53" s="27"/>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21">
       <c r="A54" s="20"/>
       <c r="B54" s="21"/>
       <c r="C54" s="20"/>
@@ -3872,20 +3892,20 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K3" r:id="rId1"/>
-    <hyperlink ref="K4" r:id="rId2"/>
-    <hyperlink ref="K5" r:id="rId3"/>
+    <hyperlink ref="K3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="K4" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="K5" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <legacyDrawing r:id="rId5"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3893,147 +3913,147 @@
     <col min="4" max="4" width="72" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="14.4" customHeight="1">
       <c r="A1" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="C1" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="D1" s="28" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" ht="14.4" customHeight="1">
       <c r="A2" s="29" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D2" s="29" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="14.4" customHeight="1">
       <c r="A3" s="29" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="29" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" ht="14.4" customHeight="1">
       <c r="A4" s="29" t="s">
         <v>37</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C4" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="29" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:4" ht="14.4" customHeight="1">
       <c r="A5" s="29" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="14.4" customHeight="1">
       <c r="A6" s="29" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="14.4" customHeight="1">
       <c r="A7" s="29" t="s">
         <v>40</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="14.4" customHeight="1">
       <c r="A8" s="29" t="s">
         <v>41</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="14.4" customHeight="1">
       <c r="A9" s="29" t="s">
         <v>42</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="14.4" customHeight="1">
       <c r="A10" s="29" t="s">
         <v>43</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="14.4" customHeight="1">
       <c r="A11" s="29" t="s">
         <v>44</v>
       </c>
@@ -4041,27 +4061,27 @@
         <v>28</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="14.4" customHeight="1">
       <c r="A12" s="29" t="s">
         <v>45</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="14.4" customHeight="1">
       <c r="A13" s="29" t="s">
         <v>46</v>
       </c>
@@ -4069,13 +4089,13 @@
         <v>28</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="14.4" customHeight="1">
       <c r="A14" s="29" t="s">
         <v>47</v>
       </c>
@@ -4083,27 +4103,27 @@
         <v>28</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="14.4" customHeight="1">
       <c r="A15" s="29" t="s">
         <v>48</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="14.4" customHeight="1">
       <c r="A16" s="29" t="s">
         <v>49</v>
       </c>
@@ -4111,98 +4131,98 @@
         <v>28</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="14.4" customHeight="1">
       <c r="A17" s="29" t="s">
         <v>50</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="14.4" customHeight="1">
       <c r="A18" s="29" t="s">
         <v>51</v>
       </c>
       <c r="B18" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:4" ht="14.4" customHeight="1">
       <c r="A19" s="29" t="s">
         <v>52</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C19" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="29" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:4" ht="14.4" customHeight="1">
       <c r="A20" s="29" t="s">
         <v>53</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="14.4" customHeight="1">
       <c r="A21" s="29" t="s">
         <v>54</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="14.4" customHeight="1">
       <c r="A22" s="29" t="s">
         <v>55</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C22" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="29" t="s">
         <v>102</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>105</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>